<commit_message>
Initial commit - update
</commit_message>
<xml_diff>
--- a/EID Roster 2026.xlsx
+++ b/EID Roster 2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MNABIL\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\moody\Downloads\whatsapp-bot - EN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF1FCD53-3A8D-46B4-BE75-3605C80600CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18790751-45D5-4FEC-89AE-433245FF3293}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="61440" windowHeight="20340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EID" sheetId="8" r:id="rId1"/>
@@ -31,9 +31,6 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -104,9 +101,6 @@
     <t>Saad Marwan</t>
   </si>
   <si>
-    <t xml:space="preserve">Mohamed Alkhatabi </t>
-  </si>
-  <si>
     <t xml:space="preserve">ziyad al zahrani </t>
   </si>
   <si>
@@ -210,9 +204,6 @@
     <t>Yasser Mattiri</t>
   </si>
   <si>
-    <t>Abdulmajed Othman</t>
-  </si>
-  <si>
     <t>Meshari Alharithi</t>
   </si>
   <si>
@@ -280,6 +271,12 @@
   </si>
   <si>
     <t>14:00 PM - 20:00 PM</t>
+  </si>
+  <si>
+    <t>Abdulmajeed Othman</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mohammed Alkhattabi </t>
   </si>
 </sst>
 </file>
@@ -1372,7 +1369,7 @@
         <v>45735</v>
       </c>
       <c r="H1" s="23" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I1" s="2">
         <v>45737</v>
@@ -1576,22 +1573,22 @@
         <v>1</v>
       </c>
       <c r="B3" s="41" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C3" s="39" t="s">
         <v>10</v>
       </c>
       <c r="D3" s="40" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E3" s="40" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F3" s="40" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G3" s="40" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>14</v>
@@ -1600,7 +1597,7 @@
         <v>14</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K3" s="3" t="s">
         <v>14</v>
@@ -1689,22 +1686,22 @@
         <v>2</v>
       </c>
       <c r="B4" s="41" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D4" s="24" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E4" s="24" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G4" s="24" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H4" s="26" t="s">
         <v>10</v>
@@ -1802,22 +1799,22 @@
         <v>3</v>
       </c>
       <c r="B5" s="41" t="s">
-        <v>21</v>
+        <v>79</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F5" s="26" t="s">
         <v>10</v>
       </c>
       <c r="G5" s="24" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H5" s="24" t="s">
         <v>17</v>
@@ -1835,10 +1832,10 @@
         <v>17</v>
       </c>
       <c r="M5" s="24" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="N5" s="24" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="O5" s="24" t="s">
         <v>17</v>
@@ -1847,13 +1844,13 @@
         <v>17</v>
       </c>
       <c r="Q5" s="26" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="R5" s="26" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="S5" s="26" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="T5" s="26" t="s">
         <v>10</v>
@@ -1918,19 +1915,19 @@
         <v>11</v>
       </c>
       <c r="C6" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G6" s="3" t="s">
         <v>70</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>72</v>
       </c>
       <c r="H6" s="26" t="s">
         <v>10</v>
@@ -2031,16 +2028,16 @@
         <v>16</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G7" s="26" t="s">
         <v>10</v>
@@ -2144,19 +2141,19 @@
         <v>20</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="H8" s="31" t="s">
         <v>13</v>
@@ -2183,7 +2180,7 @@
         <v>13</v>
       </c>
       <c r="P8" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="Q8" s="26" t="s">
         <v>10</v>
@@ -2257,25 +2254,25 @@
         <v>18</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D9" s="29" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G9" s="29" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H9" s="29" t="s">
         <v>12</v>
       </c>
       <c r="I9" s="29" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="J9" s="29" t="s">
         <v>12</v>
@@ -2317,7 +2314,7 @@
         <v>14</v>
       </c>
       <c r="W9" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="X9" s="3" t="s">
         <v>14</v>
@@ -2329,37 +2326,37 @@
         <v>14</v>
       </c>
       <c r="AA9" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AB9" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AC9" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AD9" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AE9" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AF9" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AG9" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AH9" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AI9" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AJ9" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AK9" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:37" x14ac:dyDescent="0.25">
@@ -2367,25 +2364,25 @@
         <v>8</v>
       </c>
       <c r="B10" s="41" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C10" s="40" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D10" s="40" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E10" s="40" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F10" s="40" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G10" s="40" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H10" s="29" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="I10" s="29" t="s">
         <v>12</v>
@@ -2409,7 +2406,7 @@
         <v>10</v>
       </c>
       <c r="P10" s="26" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="Q10" s="3" t="s">
         <v>14</v>
@@ -2480,13 +2477,13 @@
         <v>9</v>
       </c>
       <c r="B11" s="41" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D11" s="29" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E11" s="26" t="s">
         <v>10</v>
@@ -2531,14 +2528,14 @@
         <v>12</v>
       </c>
       <c r="S11" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="T11" s="26" t="s">
+        <v>10</v>
+      </c>
+      <c r="U11" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="T11" s="26" t="s">
-        <v>10</v>
-      </c>
-      <c r="U11" s="26" t="s">
-        <v>70</v>
-      </c>
       <c r="V11" s="3" t="s">
         <v>14</v>
       </c>
@@ -2552,13 +2549,13 @@
         <v>12</v>
       </c>
       <c r="Z11" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="AA11" s="26" t="s">
+        <v>10</v>
+      </c>
+      <c r="AB11" s="26" t="s">
         <v>68</v>
-      </c>
-      <c r="AA11" s="26" t="s">
-        <v>10</v>
-      </c>
-      <c r="AB11" s="26" t="s">
-        <v>70</v>
       </c>
       <c r="AC11" s="3" t="s">
         <v>14</v>
@@ -2593,10 +2590,10 @@
         <v>10</v>
       </c>
       <c r="B12" s="41" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C12" s="29" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D12" s="26" t="s">
         <v>10</v>
@@ -2605,10 +2602,10 @@
         <v>10</v>
       </c>
       <c r="F12" s="29" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G12" s="29" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H12" s="31" t="s">
         <v>13</v>
@@ -2706,22 +2703,22 @@
         <v>11</v>
       </c>
       <c r="B13" s="41" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C13" s="26" t="s">
         <v>10</v>
       </c>
       <c r="D13" s="29" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E13" s="29" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F13" s="29" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G13" s="29" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H13" s="26" t="s">
         <v>10</v>
@@ -2748,31 +2745,31 @@
         <v>13</v>
       </c>
       <c r="P13" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="Q13" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R13" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="S13" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="T13" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="U13" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="V13" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="W13" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="X13" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="Y13" s="3" t="s">
         <v>14</v>
@@ -2819,25 +2816,25 @@
         <v>12</v>
       </c>
       <c r="B14" s="41" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D14" s="29" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E14" s="29" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F14" s="29" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G14" s="26" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H14" s="26" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I14" s="31" t="s">
         <v>13</v>
@@ -2891,13 +2888,13 @@
         <v>17</v>
       </c>
       <c r="Z14" s="24" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="AA14" s="26" t="s">
         <v>10</v>
       </c>
       <c r="AB14" s="26" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="AC14" s="29" t="s">
         <v>12</v>
@@ -2932,7 +2929,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="41" t="s">
-        <v>56</v>
+        <v>78</v>
       </c>
       <c r="C15" s="26" t="s">
         <v>10</v>
@@ -2941,16 +2938,16 @@
         <v>10</v>
       </c>
       <c r="E15" s="29" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F15" s="29" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G15" s="26" t="s">
         <v>10</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>14</v>
@@ -2968,19 +2965,19 @@
         <v>14</v>
       </c>
       <c r="N15" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="O15" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="P15" s="26" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="Q15" s="26" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="R15" s="26" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="S15" s="29" t="s">
         <v>12</v>
@@ -3048,7 +3045,7 @@
         <v>15</v>
       </c>
       <c r="C16" s="24" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D16" s="26" t="s">
         <v>10</v>
@@ -3057,10 +3054,10 @@
         <v>10</v>
       </c>
       <c r="F16" s="24" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="H16" s="31" t="s">
         <v>13</v>
@@ -3158,16 +3155,16 @@
         <v>15</v>
       </c>
       <c r="B17" s="41" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C17" s="29" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D17" s="31" t="s">
         <v>13</v>
       </c>
       <c r="E17" s="29" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F17" s="26" t="s">
         <v>10</v>
@@ -3188,82 +3185,82 @@
         <v>13</v>
       </c>
       <c r="L17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="M17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="O17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="P17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="Q17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="S17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="T17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="U17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="V17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="W17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="X17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="Y17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="Z17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AA17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AB17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AC17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AD17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AE17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AF17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AG17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AH17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AI17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AJ17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AK17" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3274,76 +3271,76 @@
         <v>19</v>
       </c>
       <c r="C18" s="29" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F18" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G18" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H18" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J18" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="K18" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="L18" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="M18" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N18" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="O18" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="P18" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="Q18" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R18" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="S18" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="T18" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="U18" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="V18" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="W18" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="X18" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="Y18" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="Z18" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AA18" s="3" t="s">
         <v>14</v>
@@ -3424,27 +3421,27 @@
         <v>14</v>
       </c>
       <c r="C20" s="3">
-        <f>COUNTIF(C4:C19,"M")</f>
+        <f t="shared" ref="C20:H20" si="0">COUNTIF(C4:C19,"M")</f>
         <v>0</v>
       </c>
       <c r="D20" s="3">
-        <f>COUNTIF(D4:D19,"M")</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="E20" s="3">
-        <f>COUNTIF(E4:E19,"M")</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F20" s="3">
-        <f>COUNTIF(F4:F19,"M")</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G20" s="3">
-        <f>COUNTIF(G4:G19,"M")</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H20" s="3">
-        <f>COUNTIF(H4:H19,"M")</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I20" s="3">
@@ -3475,86 +3472,86 @@
         <v>3</v>
       </c>
       <c r="Q20" s="3">
-        <f>COUNTIF(Q4:Q19,"M")</f>
+        <f t="shared" ref="Q20:V20" si="1">COUNTIF(Q4:Q19,"M")</f>
         <v>6</v>
       </c>
       <c r="R20" s="3">
-        <f>COUNTIF(R4:R19,"M")</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="S20" s="3">
-        <f>COUNTIF(S4:S19,"M")</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="T20" s="3">
-        <f>COUNTIF(T4:T19,"M")</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="U20" s="3">
-        <f>COUNTIF(U4:U19,"M")</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="V20" s="3">
-        <f>COUNTIF(V4:V19,"M")</f>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="W20" s="3">
         <v>3</v>
       </c>
       <c r="X20" s="3">
-        <f>COUNTIF(X4:X19,"M")</f>
+        <f t="shared" ref="X20:AK20" si="2">COUNTIF(X4:X19,"M")</f>
         <v>7</v>
       </c>
       <c r="Y20" s="3">
-        <f>COUNTIF(Y4:Y19,"M")</f>
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
       <c r="Z20" s="3">
-        <f>COUNTIF(Z4:Z19,"M")</f>
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
       <c r="AA20" s="3">
-        <f>COUNTIF(AA4:AA19,"M")</f>
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
       <c r="AB20" s="3">
-        <f>COUNTIF(AB4:AB19,"M")</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="AC20" s="3">
-        <f>COUNTIF(AC4:AC19,"M")</f>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="AD20" s="3">
-        <f>COUNTIF(AD4:AD19,"M")</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="AE20" s="3">
-        <f>COUNTIF(AE4:AE19,"M")</f>
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
       <c r="AF20" s="3">
-        <f>COUNTIF(AF4:AF19,"M")</f>
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
       <c r="AG20" s="3">
-        <f>COUNTIF(AG4:AG19,"M")</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="AH20" s="3">
-        <f>COUNTIF(AH4:AH19,"M")</f>
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
       <c r="AI20" s="3">
-        <f>COUNTIF(AI4:AI19,"M")</f>
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
       <c r="AJ20" s="3">
-        <f>COUNTIF(AJ4:AJ19,"M")</f>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="AK20" s="3">
-        <f>COUNTIF(AK4:AK19,"M")</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
     </row>
@@ -3564,143 +3561,143 @@
         <v>9</v>
       </c>
       <c r="C21" s="34">
-        <f>COUNTIF(C5:C19,"B")</f>
+        <f t="shared" ref="C21:AK21" si="3">COUNTIF(C5:C19,"B")</f>
         <v>0</v>
       </c>
       <c r="D21" s="34">
-        <f>COUNTIF(D5:D19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="E21" s="34">
-        <f>COUNTIF(E5:E19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F21" s="34">
-        <f>COUNTIF(F5:F19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="G21" s="34">
-        <f>COUNTIF(G5:G19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H21" s="34">
-        <f>COUNTIF(H5:H19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="I21" s="34">
-        <f>COUNTIF(I5:I19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J21" s="34">
-        <f>COUNTIF(J5:J19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="K21" s="34">
-        <f>COUNTIF(K5:K19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L21" s="34">
-        <f>COUNTIF(L5:L19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="M21" s="34">
-        <f>COUNTIF(M5:M19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="N21" s="34">
-        <f>COUNTIF(N5:N19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="O21" s="34">
-        <f>COUNTIF(O5:O19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="P21" s="34">
-        <f>COUNTIF(P5:P19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="Q21" s="34">
-        <f>COUNTIF(Q5:Q19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="R21" s="34">
-        <f>COUNTIF(R5:R19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="S21" s="34">
-        <f>COUNTIF(S5:S19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="T21" s="34">
-        <f>COUNTIF(T5:T19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="U21" s="34">
-        <f>COUNTIF(U5:U19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="V21" s="34">
-        <f>COUNTIF(V5:V19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="W21" s="34">
-        <f>COUNTIF(W5:W19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="X21" s="34">
-        <f>COUNTIF(X5:X19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="Y21" s="34">
-        <f>COUNTIF(Y5:Y19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="Z21" s="34">
-        <f>COUNTIF(Z5:Z19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AA21" s="34">
-        <f>COUNTIF(AA5:AA19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AB21" s="34">
-        <f>COUNTIF(AB5:AB19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AC21" s="34">
-        <f>COUNTIF(AC5:AC19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AD21" s="34">
-        <f>COUNTIF(AD5:AD19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AE21" s="34">
-        <f>COUNTIF(AE5:AE19,"B")</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="AF21" s="34">
-        <f>COUNTIF(AF5:AF19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AG21" s="34">
-        <f>COUNTIF(AG5:AG19,"B")</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="AH21" s="34">
-        <f>COUNTIF(AH5:AH19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AI21" s="34">
-        <f>COUNTIF(AI5:AI19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AJ21" s="34">
-        <f>COUNTIF(AJ5:AJ19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AK21" s="34">
-        <f>COUNTIF(AK5:AK19,"B")</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -3710,35 +3707,35 @@
         <v>12</v>
       </c>
       <c r="C22" s="29">
-        <f>COUNTIF(C4:C19,"E")</f>
+        <f t="shared" ref="C22:J22" si="4">COUNTIF(C4:C19,"E")</f>
         <v>0</v>
       </c>
       <c r="D22" s="29">
-        <f>COUNTIF(D4:D19,"E")</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="E22" s="29">
-        <f>COUNTIF(E4:E19,"E")</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="F22" s="29">
-        <f>COUNTIF(F4:F19,"E")</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="G22" s="29">
-        <f>COUNTIF(G4:G19,"E")</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H22" s="29">
-        <f>COUNTIF(H4:H19,"E")</f>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I22" s="29">
-        <f>COUNTIF(I4:I19,"E")</f>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="J22" s="29">
-        <f>COUNTIF(J4:J19,"E")</f>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="K22" s="29">
@@ -3748,103 +3745,103 @@
         <v>1</v>
       </c>
       <c r="M22" s="29">
-        <f>COUNTIF(M4:M19,"E")</f>
+        <f t="shared" ref="M22:AK22" si="5">COUNTIF(M4:M19,"E")</f>
         <v>2</v>
       </c>
       <c r="N22" s="29">
-        <f>COUNTIF(N4:N19,"E")</f>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="O22" s="29">
-        <f>COUNTIF(O4:O19,"E")</f>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="P22" s="29">
-        <f>COUNTIF(P4:P19,"E")</f>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="Q22" s="29">
-        <f>COUNTIF(Q4:Q19,"E")</f>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="R22" s="29">
-        <f>COUNTIF(R4:R19,"E")</f>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="S22" s="29">
-        <f>COUNTIF(S4:S19,"E")</f>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="T22" s="29">
-        <f>COUNTIF(T4:T19,"E")</f>
+        <f t="shared" si="5"/>
         <v>3</v>
       </c>
       <c r="U22" s="29">
-        <f>COUNTIF(U4:U19,"E")</f>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="V22" s="29">
-        <f>COUNTIF(V4:V19,"E")</f>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="W22" s="29">
-        <f>COUNTIF(W4:W19,"E")</f>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="X22" s="29">
-        <f>COUNTIF(X4:X19,"E")</f>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="Y22" s="29">
-        <f>COUNTIF(Y4:Y19,"E")</f>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="Z22" s="29">
-        <f>COUNTIF(Z4:Z19,"E")</f>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AA22" s="29">
-        <f>COUNTIF(AA4:AA19,"E")</f>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="AB22" s="29">
-        <f>COUNTIF(AB4:AB19,"E")</f>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="AC22" s="29">
-        <f>COUNTIF(AC4:AC19,"E")</f>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="AD22" s="29">
-        <f>COUNTIF(AD4:AD19,"E")</f>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="AE22" s="29">
-        <f>COUNTIF(AE4:AE19,"E")</f>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="AF22" s="29">
-        <f>COUNTIF(AF4:AF19,"E")</f>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="AG22" s="29">
-        <f>COUNTIF(AG4:AG19,"E")</f>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="AH22" s="29">
-        <f>COUNTIF(AH4:AH19,"E")</f>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="AI22" s="29">
-        <f>COUNTIF(AI4:AI19,"E")</f>
+        <f t="shared" si="5"/>
         <v>3</v>
       </c>
       <c r="AJ22" s="29">
-        <f>COUNTIF(AJ4:AJ19,"E")</f>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="AK22" s="29">
-        <f>COUNTIF(AK4:AK19,"E")</f>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
     </row>
@@ -3870,126 +3867,126 @@
         <v>0</v>
       </c>
       <c r="G23" s="38">
-        <f t="shared" ref="G23:AK23" si="0">COUNTIF(G4:G19,"N")</f>
+        <f t="shared" ref="G23:AK23" si="6">COUNTIF(G4:G19,"N")</f>
         <v>0</v>
       </c>
       <c r="H23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="I23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="J23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="K23" s="38">
         <v>1</v>
       </c>
       <c r="L23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="M23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="N23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="O23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="P23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="Q23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="R23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="S23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="T23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="U23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="V23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="W23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="X23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="Y23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="Z23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AA23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AB23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AC23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AD23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AE23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AF23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AG23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AH23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AI23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AJ23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="AK23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
     </row>
@@ -3999,7 +3996,7 @@
         <v>14</v>
       </c>
       <c r="B25" s="45" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
@@ -4014,7 +4011,7 @@
         <v>12</v>
       </c>
       <c r="B26" s="47" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G26" s="8"/>
       <c r="H26" s="8"/>
@@ -4029,7 +4026,7 @@
         <v>17</v>
       </c>
       <c r="B27" s="43" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G27" s="8"/>
       <c r="H27" s="8"/>
@@ -4044,7 +4041,7 @@
         <v>9</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G28" s="8"/>
       <c r="H28" s="8"/>
@@ -4054,15 +4051,15 @@
       <c r="L28" s="8"/>
       <c r="M28" s="8"/>
       <c r="N28" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="29" spans="1:37" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29" s="10" t="s">
         <v>29</v>
-      </c>
-      <c r="B29" s="10" t="s">
-        <v>30</v>
       </c>
       <c r="G29" s="8"/>
       <c r="H29" s="8"/>
@@ -4074,10 +4071,10 @@
     </row>
     <row r="30" spans="1:37" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30" s="10" t="s">
         <v>31</v>
-      </c>
-      <c r="B30" s="10" t="s">
-        <v>32</v>
       </c>
       <c r="G30" s="8"/>
       <c r="H30" s="8"/>
@@ -4089,10 +4086,10 @@
     </row>
     <row r="31" spans="1:37" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B31" s="10" t="s">
         <v>33</v>
-      </c>
-      <c r="B31" s="10" t="s">
-        <v>34</v>
       </c>
       <c r="G31" s="8"/>
       <c r="H31" s="8"/>
@@ -4107,7 +4104,7 @@
         <v>13</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G32" s="8"/>
       <c r="H32" s="8"/>
@@ -4119,10 +4116,10 @@
     </row>
     <row r="33" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" s="10" t="s">
         <v>36</v>
-      </c>
-      <c r="B33" s="10" t="s">
-        <v>37</v>
       </c>
       <c r="G33" s="8"/>
       <c r="H33" s="8"/>
@@ -4134,10 +4131,10 @@
     </row>
     <row r="34" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B34" s="10" t="s">
         <v>38</v>
-      </c>
-      <c r="B34" s="10" t="s">
-        <v>39</v>
       </c>
       <c r="G34" s="8"/>
       <c r="H34" s="8"/>
@@ -4149,10 +4146,10 @@
     </row>
     <row r="35" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B35" s="10" t="s">
         <v>40</v>
-      </c>
-      <c r="B35" s="10" t="s">
-        <v>41</v>
       </c>
       <c r="G35" s="8"/>
       <c r="H35" s="8"/>
@@ -4167,7 +4164,7 @@
         <v>10</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G36" s="8"/>
       <c r="H36" s="8"/>
@@ -4179,10 +4176,10 @@
     </row>
     <row r="37" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="B37" s="10" t="s">
         <v>43</v>
-      </c>
-      <c r="B37" s="10" t="s">
-        <v>44</v>
       </c>
       <c r="G37" s="8"/>
       <c r="H37" s="8"/>
@@ -4194,10 +4191,10 @@
     </row>
     <row r="38" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="B38" s="10" t="s">
         <v>45</v>
-      </c>
-      <c r="B38" s="10" t="s">
-        <v>46</v>
       </c>
       <c r="G38" s="8"/>
       <c r="H38" s="8"/>
@@ -4209,10 +4206,10 @@
     </row>
     <row r="39" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="B39" s="10" t="s">
         <v>47</v>
-      </c>
-      <c r="B39" s="10" t="s">
-        <v>48</v>
       </c>
       <c r="G39" s="8"/>
       <c r="H39" s="8"/>
@@ -4224,10 +4221,10 @@
     </row>
     <row r="40" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="B40" s="10" t="s">
         <v>49</v>
-      </c>
-      <c r="B40" s="10" t="s">
-        <v>50</v>
       </c>
       <c r="G40" s="8"/>
       <c r="H40" s="8"/>
@@ -4239,10 +4236,10 @@
     </row>
     <row r="41" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="21" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G41" s="8"/>
       <c r="H41" s="8"/>
@@ -4254,10 +4251,10 @@
     </row>
     <row r="42" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="22" t="s">
+        <v>51</v>
+      </c>
+      <c r="B42" s="10" t="s">
         <v>52</v>
-      </c>
-      <c r="B42" s="10" t="s">
-        <v>53</v>
       </c>
       <c r="G42" s="8"/>
       <c r="H42" s="8"/>

</xml_diff>

<commit_message>
Add shift editing per employee and auto in-charge by priority
- Each employee row has an Edit button to change their shift
- In-charge auto-assigned by priority: Salem > Saad > Mostafa >
  Islam > Alamoudi > Moayad > Ziyad > Mohammed > Suhaib > Hatem >
  Yasser > Meshari > Abdulmajeed > Haitham
- Manual override still available via dropdown
- Removed Hotel In-Charge tab

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/EID Roster 2026.xlsx
+++ b/EID Roster 2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\moody\Downloads\whatsapp-bot - EN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18790751-45D5-4FEC-89AE-433245FF3293}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4EFBCF5-778D-4838-A7FF-53755A56CCA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="61440" windowHeight="20340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="77040" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EID" sheetId="8" r:id="rId1"/>
@@ -1644,41 +1644,41 @@
       <c r="Y3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="Z3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="AA3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="AB3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="AC3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="AD3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="AE3" s="26" t="s">
-        <v>10</v>
-      </c>
-      <c r="AF3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="AG3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="AH3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="AI3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="AJ3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="AK3" s="3" t="s">
-        <v>14</v>
+      <c r="Z3" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="AA3" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="AB3" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="AC3" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="AD3" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="AE3" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF3" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="AG3" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="AH3" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="AI3" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="AJ3" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="AK3" s="30" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1989,8 +1989,8 @@
       <c r="AA6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="AB6" s="29" t="s">
-        <v>12</v>
+      <c r="AB6" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="AC6" s="26" t="s">
         <v>10</v>
@@ -2209,8 +2209,8 @@
       <c r="Y8" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="Z8" s="3" t="s">
-        <v>14</v>
+      <c r="Z8" s="17" t="s">
+        <v>42</v>
       </c>
       <c r="AA8" s="3" t="s">
         <v>14</v>
@@ -2780,8 +2780,8 @@
       <c r="AA13" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="AB13" s="3" t="s">
-        <v>14</v>
+      <c r="AB13" s="29" t="s">
+        <v>12</v>
       </c>
       <c r="AC13" s="26" t="s">
         <v>10</v>
@@ -2924,7 +2924,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:37" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="28">
         <v>13</v>
       </c>
@@ -2997,8 +2997,8 @@
       <c r="X15" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="Y15" s="3" t="s">
-        <v>14</v>
+      <c r="Y15" s="17" t="s">
+        <v>42</v>
       </c>
       <c r="Z15" s="3" t="s">
         <v>14</v>
@@ -3504,11 +3504,11 @@
       </c>
       <c r="Y20" s="3">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Z20" s="3">
         <f t="shared" si="2"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AA20" s="3">
         <f t="shared" si="2"/>

</xml_diff>